<commit_message>
Populate Stage 4 live market data and document sources
</commit_message>
<xml_diff>
--- a/models/builds/2026-08-08-Vuong-tech-services-model.xlsx
+++ b/models/builds/2026-08-08-Vuong-tech-services-model.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vuong\OneDrive\Documents\GitHub\Timmy Vuong\models\builds\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CE74DC1-755A-4EEB-AC75-D7C1CD1AE216}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8753436-C22A-4313-8ADE-BFB3844813CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2895" yWindow="375" windowWidth="23820" windowHeight="19890" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2895" yWindow="375" windowWidth="23820" windowHeight="19890" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cover" sheetId="1" r:id="rId1"/>
@@ -106,9 +106,6 @@
     <t>Market data</t>
   </si>
   <si>
-    <t>Indicative</t>
-  </si>
-  <si>
     <t>Replace with sourced live values in Stage 4</t>
   </si>
   <si>
@@ -187,9 +184,6 @@
     <t>Reference payoff; does not protect a EUR receivable from euro weakness.</t>
   </si>
   <si>
-    <t>PRELIMINARY STAGE 3 MODEL — The workbook is fully formula-driven, but S0_in, R_USD, R_FC, K_PUT, and K_CALL are indicative assumptions. Replace and source them in Stage 4 before making a hedge recommendation.</t>
-  </si>
-  <si>
     <t>Legend &amp; Key</t>
   </si>
   <si>
@@ -385,48 +379,27 @@
     <t>USD per EUR</t>
   </si>
   <si>
-    <t>Stage 3 modeling assumption; replace in Stage 4</t>
-  </si>
-  <si>
     <t>One-year EUR/USD forward rate</t>
   </si>
   <si>
     <t>Assigned / indicative</t>
   </si>
   <si>
-    <t>Scenario 3 forward quote; replace with live Stage 4 quote</t>
-  </si>
-  <si>
     <t>Annual USD interest rate</t>
   </si>
   <si>
     <t>Decimal annual rate</t>
   </si>
   <si>
-    <t>Stage 3 modeling assumption</t>
-  </si>
-  <si>
     <t>Annual EUR interest rate</t>
   </si>
   <si>
-    <t>Indicative / calibrated</t>
-  </si>
-  <si>
-    <t>Calibrated to S0_in, R_USD, and F0_in for parity demonstration</t>
-  </si>
-  <si>
     <t>EUR put-option strike rate</t>
   </si>
   <si>
-    <t>Near-the-money illustrative strike; replace in Stage 4</t>
-  </si>
-  <si>
     <t>EUR call-option strike rate</t>
   </si>
   <si>
-    <t>Illustrative call strike; replace in Stage 4</t>
-  </si>
-  <si>
     <t>EUR put-option premium</t>
   </si>
   <si>
@@ -809,6 +782,33 @@
   </si>
   <si>
     <t>Build contract and audit requirements.</t>
+  </si>
+  <si>
+    <t>Live / sourced</t>
+  </si>
+  <si>
+    <t>PRELIMINARY STAGE 3 MODEL —STAGE 4 LIVE MARKET DATA — Spot and one-year rates sourced as of 2026-08-06/07; F0_in is CIP-implied; scenario option premiums were retained as assumptions.</t>
+  </si>
+  <si>
+    <t>ECB EUR/USD reference rate, 2026-08-07</t>
+  </si>
+  <si>
+    <t>CIP-implied</t>
+  </si>
+  <si>
+    <t>Calculated from live spot and one-year USD/EUR rates</t>
+  </si>
+  <si>
+    <t>FRED DGS1 one-year Treasury rate, 2026-08-06</t>
+  </si>
+  <si>
+    <t>ECB AAA euro-area one-year yield, 2026-08-06</t>
+  </si>
+  <si>
+    <t>Stage 4 assumption</t>
+  </si>
+  <si>
+    <t>Set equal to live spot as an at-the-money strike</t>
   </si>
 </sst>
 </file>
@@ -1248,9 +1248,13 @@
     <xf numFmtId="1" fontId="6" fillId="6" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1269,9 +1273,6 @@
     <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -1299,7 +1300,6 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1469,37 +1469,37 @@
                 <c:formatCode>\$#,##0;[Red]\(\$#,##0\);\-</c:formatCode>
                 <c:ptCount val="11"/>
                 <c:pt idx="0">
-                  <c:v>12825000</c:v>
+                  <c:v>13697812.499999998</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>12960000</c:v>
+                  <c:v>13841999.999999998</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>13095000.000000002</c:v>
+                  <c:v>13986187.5</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>13230000</c:v>
+                  <c:v>14130375</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>13365000.000000002</c:v>
+                  <c:v>14274562.499999998</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>13500000</c:v>
+                  <c:v>14418750</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>13635000</c:v>
+                  <c:v>14562937.5</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>13770000.000000002</c:v>
+                  <c:v>14707124.999999998</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>13905000</c:v>
+                  <c:v>14851312.5</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>14040000.000000002</c:v>
+                  <c:v>14995500</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>14175000.000000002</c:v>
+                  <c:v>15139687.500000002</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1568,37 +1568,37 @@
                 <c:formatCode>\$#,##0;[Red]\(\$#,##0\);\-</c:formatCode>
                 <c:ptCount val="11"/>
                 <c:pt idx="0">
-                  <c:v>13637500</c:v>
+                  <c:v>14633512.500000002</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>13637500</c:v>
+                  <c:v>14633512.500000002</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>13637500</c:v>
+                  <c:v>14633512.500000002</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>13637500</c:v>
+                  <c:v>14633512.500000002</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>13637500</c:v>
+                  <c:v>14633512.500000002</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>13637500</c:v>
+                  <c:v>14633512.500000002</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>13637500</c:v>
+                  <c:v>14633512.500000002</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>13637500</c:v>
+                  <c:v>14633512.500000002</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>13637500</c:v>
+                  <c:v>14633512.500000002</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>13637500</c:v>
+                  <c:v>14633512.500000002</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>13637500</c:v>
+                  <c:v>14633512.500000002</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1667,37 +1667,37 @@
                 <c:formatCode>\$#,##0;[Red]\(\$#,##0\);\-</c:formatCode>
                 <c:ptCount val="11"/>
                 <c:pt idx="0">
-                  <c:v>13637499.999999998</c:v>
+                  <c:v>14633514.240847424</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>13637499.999999998</c:v>
+                  <c:v>14633514.240847424</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>13637499.999999998</c:v>
+                  <c:v>14633514.240847424</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>13637499.999999998</c:v>
+                  <c:v>14633514.240847424</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>13637499.999999998</c:v>
+                  <c:v>14633514.240847424</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>13637499.999999998</c:v>
+                  <c:v>14633514.240847424</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>13637499.999999998</c:v>
+                  <c:v>14633514.240847424</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>13637499.999999998</c:v>
+                  <c:v>14633514.240847424</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>13637499.999999998</c:v>
+                  <c:v>14633514.240847424</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>13637499.999999998</c:v>
+                  <c:v>14633514.240847424</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>13637499.999999998</c:v>
+                  <c:v>14633514.240847424</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1766,37 +1766,37 @@
                 <c:formatCode>\$#,##0;[Red]\(\$#,##0\);\-</c:formatCode>
                 <c:ptCount val="11"/>
                 <c:pt idx="0">
-                  <c:v>13162500</c:v>
+                  <c:v>14206250</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>13162500</c:v>
+                  <c:v>14206250</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>13162500</c:v>
+                  <c:v>14206250</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>13162500</c:v>
+                  <c:v>14206250</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>13162500</c:v>
+                  <c:v>14206250</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>13287500</c:v>
+                  <c:v>14206250</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>13422500</c:v>
+                  <c:v>14350437.5</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>13557500.000000002</c:v>
+                  <c:v>14494624.999999998</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>13692500</c:v>
+                  <c:v>14638812.5</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>13827500.000000002</c:v>
+                  <c:v>14783000</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>13962500.000000002</c:v>
+                  <c:v>14927187.500000002</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1865,37 +1865,37 @@
                 <c:formatCode>\$#,##0;[Red]\(\$#,##0\);\-</c:formatCode>
                 <c:ptCount val="11"/>
                 <c:pt idx="0">
-                  <c:v>12550000</c:v>
+                  <c:v>13422812.499999998</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>12685000</c:v>
+                  <c:v>13566999.999999998</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>12820000.000000002</c:v>
+                  <c:v>13711187.5</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>12955000</c:v>
+                  <c:v>13855375</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>13090000.000000002</c:v>
+                  <c:v>13999562.499999998</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>13225000</c:v>
+                  <c:v>14143750</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>13360000</c:v>
+                  <c:v>14432125</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>13495000.000000002</c:v>
+                  <c:v>14720499.999999996</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>13660000</c:v>
+                  <c:v>15008875</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>13930000.000000004</c:v>
+                  <c:v>15297250</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>14200000.000000002</c:v>
+                  <c:v>15585625.000000004</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2269,30 +2269,30 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="30" customHeight="1">
-      <c r="A1" s="46" t="s">
+      <c r="A1" s="47" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="46"/>
-      <c r="C1" s="46"/>
-      <c r="D1" s="46"/>
-      <c r="E1" s="46"/>
-      <c r="F1" s="46"/>
-      <c r="G1" s="46"/>
-      <c r="H1" s="46"/>
-      <c r="I1" s="46"/>
-      <c r="J1" s="46"/>
+      <c r="B1" s="47"/>
+      <c r="C1" s="47"/>
+      <c r="D1" s="47"/>
+      <c r="E1" s="47"/>
+      <c r="F1" s="47"/>
+      <c r="G1" s="47"/>
+      <c r="H1" s="47"/>
+      <c r="I1" s="47"/>
+      <c r="J1" s="47"/>
     </row>
     <row r="2" spans="1:10" ht="30" customHeight="1">
-      <c r="A2" s="46"/>
-      <c r="B2" s="46"/>
-      <c r="C2" s="46"/>
-      <c r="D2" s="46"/>
-      <c r="E2" s="46"/>
-      <c r="F2" s="46"/>
-      <c r="G2" s="46"/>
-      <c r="H2" s="46"/>
-      <c r="I2" s="46"/>
-      <c r="J2" s="46"/>
+      <c r="A2" s="47"/>
+      <c r="B2" s="47"/>
+      <c r="C2" s="47"/>
+      <c r="D2" s="47"/>
+      <c r="E2" s="47"/>
+      <c r="F2" s="47"/>
+      <c r="G2" s="47"/>
+      <c r="H2" s="47"/>
+      <c r="I2" s="47"/>
+      <c r="J2" s="47"/>
     </row>
     <row r="4" spans="1:10" ht="21.95" customHeight="1">
       <c r="A4" s="40" t="s">
@@ -2308,11 +2308,11 @@
         <f>Checks!B3</f>
         <v>PASS</v>
       </c>
-      <c r="H4" s="47" t="s">
+      <c r="H4" s="49" t="s">
         <v>4</v>
       </c>
-      <c r="I4" s="48"/>
-      <c r="J4" s="49"/>
+      <c r="I4" s="50"/>
+      <c r="J4" s="51"/>
     </row>
     <row r="5" spans="1:10" ht="15">
       <c r="A5" s="41" t="s">
@@ -2359,86 +2359,86 @@
         <v>16</v>
       </c>
       <c r="I7" s="15" t="s">
+        <v>243</v>
+      </c>
+      <c r="J7" s="3" t="s">
         <v>17</v>
-      </c>
-      <c r="J7" s="3" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="8" spans="1:10" ht="15">
       <c r="A8" s="41" t="s">
+        <v>18</v>
+      </c>
+      <c r="B8" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="H8" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="H8" s="3" t="s">
+      <c r="I8" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="J8" s="3" t="s">
         <v>21</v>
-      </c>
-      <c r="I8" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="J8" s="3" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="9" spans="1:10" ht="15">
       <c r="A9" s="41" t="s">
+        <v>22</v>
+      </c>
+      <c r="B9" s="3" t="s">
         <v>23</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="10" spans="1:10" ht="15">
       <c r="A10" s="41" t="s">
+        <v>24</v>
+      </c>
+      <c r="B10" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="B10" s="3" t="s">
+    </row>
+    <row r="12" spans="1:10" ht="21.95" customHeight="1">
+      <c r="A12" s="49" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="12" spans="1:10" ht="21.95" customHeight="1">
-      <c r="A12" s="47" t="s">
-        <v>27</v>
-      </c>
-      <c r="B12" s="48"/>
-      <c r="C12" s="48"/>
-      <c r="D12" s="48"/>
-      <c r="E12" s="48"/>
-      <c r="F12" s="49"/>
+      <c r="B12" s="50"/>
+      <c r="C12" s="50"/>
+      <c r="D12" s="50"/>
+      <c r="E12" s="50"/>
+      <c r="F12" s="51"/>
     </row>
     <row r="13" spans="1:10" ht="15">
       <c r="A13" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B13" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B13" s="1" t="s">
+      <c r="C13" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="C13" s="1" t="s">
+      <c r="D13" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="D13" s="1" t="s">
+      <c r="E13" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="E13" s="1" t="s">
+      <c r="F13" s="1" t="s">
         <v>32</v>
-      </c>
-      <c r="F13" s="1" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="14" spans="1:10" ht="15">
       <c r="A14" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B14" s="34">
         <f>FC_AMT*S0_in</f>
-        <v>13500000</v>
+        <v>14418750</v>
       </c>
       <c r="C14" s="42">
         <f>B14/FC_AMT</f>
-        <v>1.08</v>
+        <v>1.1535</v>
       </c>
       <c r="D14" s="34">
         <f>0</f>
@@ -2449,20 +2449,20 @@
         <v>0</v>
       </c>
       <c r="F14" s="12" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="15" spans="1:10" ht="15">
       <c r="A15" s="3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B15" s="26">
         <f>'Forward Hedge'!B10</f>
-        <v>13637500</v>
+        <v>14633512.500000002</v>
       </c>
       <c r="C15" s="27">
         <f>B15/FC_AMT</f>
-        <v>1.091</v>
+        <v>1.1706810000000001</v>
       </c>
       <c r="D15" s="26">
         <f>0</f>
@@ -2470,23 +2470,23 @@
       </c>
       <c r="E15" s="26">
         <f>B15-B14</f>
-        <v>137500</v>
+        <v>214762.50000000186</v>
       </c>
       <c r="F15" s="13" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="16" spans="1:10" ht="15">
       <c r="A16" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B16" s="26">
         <f>'Money Market'!C9</f>
-        <v>13637499.999999998</v>
+        <v>14633514.240847424</v>
       </c>
       <c r="C16" s="27">
         <f>B16/FC_AMT</f>
-        <v>1.0909999999999997</v>
+        <v>1.1706811392677938</v>
       </c>
       <c r="D16" s="26">
         <f>0</f>
@@ -2494,23 +2494,23 @@
       </c>
       <c r="E16" s="26">
         <f>B16-B14</f>
-        <v>137499.99999999814</v>
+        <v>214764.24084742367</v>
       </c>
       <c r="F16" s="13" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="17" spans="1:6" ht="15">
       <c r="A17" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B17" s="26">
         <f>'Option Hedge'!B12</f>
-        <v>13287500</v>
+        <v>14206250</v>
       </c>
       <c r="C17" s="27">
         <f>B17/FC_AMT</f>
-        <v>1.0629999999999999</v>
+        <v>1.1365000000000001</v>
       </c>
       <c r="D17" s="26">
         <f>FC_AMT*PREM_PUT</f>
@@ -2521,20 +2521,20 @@
         <v>-212500</v>
       </c>
       <c r="F17" s="13" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="18" spans="1:6" ht="30">
       <c r="A18" s="3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B18" s="26">
         <f>'Option Hedge'!B19</f>
-        <v>13225000</v>
+        <v>14143750</v>
       </c>
       <c r="C18" s="27">
         <f>B18/FC_AMT</f>
-        <v>1.0580000000000001</v>
+        <v>1.1315</v>
       </c>
       <c r="D18" s="26">
         <f>FC_AMT*PREM_CALL</f>
@@ -2545,37 +2545,37 @@
         <v>-275000</v>
       </c>
       <c r="F18" s="13" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="20" spans="1:6">
-      <c r="A20" s="50" t="s">
-        <v>44</v>
-      </c>
-      <c r="B20" s="50"/>
-      <c r="C20" s="50"/>
-      <c r="D20" s="50"/>
-      <c r="E20" s="50"/>
-      <c r="F20" s="50"/>
+      <c r="A20" s="52" t="s">
+        <v>244</v>
+      </c>
+      <c r="B20" s="52"/>
+      <c r="C20" s="52"/>
+      <c r="D20" s="52"/>
+      <c r="E20" s="52"/>
+      <c r="F20" s="52"/>
     </row>
     <row r="21" spans="1:6">
-      <c r="A21" s="50"/>
-      <c r="B21" s="50"/>
-      <c r="C21" s="50"/>
-      <c r="D21" s="50"/>
-      <c r="E21" s="50"/>
-      <c r="F21" s="50"/>
+      <c r="A21" s="52"/>
+      <c r="B21" s="52"/>
+      <c r="C21" s="52"/>
+      <c r="D21" s="52"/>
+      <c r="E21" s="52"/>
+      <c r="F21" s="52"/>
     </row>
     <row r="22" spans="1:6">
-      <c r="A22" s="50"/>
-      <c r="B22" s="50"/>
-      <c r="C22" s="50"/>
-      <c r="D22" s="50"/>
-      <c r="E22" s="50"/>
-      <c r="F22" s="50"/>
+      <c r="A22" s="52"/>
+      <c r="B22" s="52"/>
+      <c r="C22" s="52"/>
+      <c r="D22" s="52"/>
+      <c r="E22" s="52"/>
+      <c r="F22" s="52"/>
     </row>
     <row r="34" spans="5:5">
-      <c r="E34" s="63"/>
+      <c r="E34" s="46"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -2604,260 +2604,260 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="30" customHeight="1">
-      <c r="A1" s="46" t="s">
-        <v>45</v>
-      </c>
-      <c r="B1" s="46"/>
-      <c r="C1" s="46"/>
-      <c r="D1" s="46"/>
-      <c r="E1" s="46"/>
-      <c r="F1" s="46"/>
+      <c r="A1" s="47" t="s">
+        <v>43</v>
+      </c>
+      <c r="B1" s="47"/>
+      <c r="C1" s="47"/>
+      <c r="D1" s="47"/>
+      <c r="E1" s="47"/>
+      <c r="F1" s="47"/>
     </row>
     <row r="2" spans="1:6" ht="30" customHeight="1">
-      <c r="A2" s="46"/>
-      <c r="B2" s="46"/>
-      <c r="C2" s="46"/>
-      <c r="D2" s="46"/>
-      <c r="E2" s="46"/>
-      <c r="F2" s="46"/>
+      <c r="A2" s="47"/>
+      <c r="B2" s="47"/>
+      <c r="C2" s="47"/>
+      <c r="D2" s="47"/>
+      <c r="E2" s="47"/>
+      <c r="F2" s="47"/>
     </row>
     <row r="4" spans="1:6" ht="21.95" customHeight="1">
-      <c r="A4" s="47" t="s">
-        <v>46</v>
-      </c>
-      <c r="B4" s="48"/>
-      <c r="C4" s="48"/>
-      <c r="D4" s="48"/>
-      <c r="E4" s="48"/>
-      <c r="F4" s="49"/>
+      <c r="A4" s="49" t="s">
+        <v>44</v>
+      </c>
+      <c r="B4" s="50"/>
+      <c r="C4" s="50"/>
+      <c r="D4" s="50"/>
+      <c r="E4" s="50"/>
+      <c r="F4" s="51"/>
     </row>
     <row r="5" spans="1:6" ht="15">
       <c r="A5" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C5" s="1" t="s">
         <v>47</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>49</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="15">
       <c r="A6" s="14" t="s">
+        <v>48</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>50</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="15">
       <c r="A7" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="C7" s="3" t="s">
         <v>53</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="15">
       <c r="A8" s="20" t="s">
+        <v>54</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C8" s="3" t="s">
         <v>56</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="15">
       <c r="A9" s="21" t="s">
+        <v>57</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="C9" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="B9" s="3" t="s">
+    </row>
+    <row r="11" spans="1:6" ht="21.95" customHeight="1">
+      <c r="A11" s="49" t="s">
         <v>60</v>
       </c>
-      <c r="C9" s="3" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" ht="21.95" customHeight="1">
-      <c r="A11" s="47" t="s">
-        <v>62</v>
-      </c>
-      <c r="B11" s="48"/>
-      <c r="C11" s="48"/>
-      <c r="D11" s="48"/>
-      <c r="E11" s="48"/>
-      <c r="F11" s="49"/>
+      <c r="B11" s="50"/>
+      <c r="C11" s="50"/>
+      <c r="D11" s="50"/>
+      <c r="E11" s="50"/>
+      <c r="F11" s="51"/>
     </row>
     <row r="12" spans="1:6" ht="15">
       <c r="A12" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="D12" s="1" t="s">
         <v>63</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="D12" s="1" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="15">
       <c r="A13" s="2" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C13" s="43">
         <f>FC_AMT</f>
         <v>12500000</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="15">
       <c r="A14" s="3" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="C14" s="27">
         <f>S0_in</f>
-        <v>1.08</v>
+        <v>1.1535</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="15">
       <c r="A15" s="3" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="C15" s="27">
         <f>F0_in</f>
-        <v>1.091</v>
+        <v>1.1706810000000001</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="16" spans="1:6" ht="15">
       <c r="A16" s="3" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C16" s="44">
         <f>R_USD</f>
-        <v>4.4999999999999998E-2</v>
+        <v>4.0599999999999997E-2</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="15">
       <c r="A17" s="3" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C17" s="44">
         <f>R_FC</f>
-        <v>3.4601911027962513E-2</v>
+        <v>2.5529E-2</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="15">
       <c r="A18" s="3" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="C18" s="27">
         <f>K_PUT</f>
-        <v>1.07</v>
+        <v>1.1535</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="15">
       <c r="A19" s="3" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="C19" s="27">
         <f>K_CALL</f>
-        <v>1.1100000000000001</v>
+        <v>1.1535</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="20" spans="1:4" ht="15">
       <c r="A20" s="3" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C20" s="27">
         <f>PREM_PUT</f>
         <v>1.7000000000000001E-2</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
     </row>
     <row r="21" spans="1:4" ht="15">
       <c r="A21" s="3" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C21" s="27">
         <f>PREM_CALL</f>
         <v>2.1999999999999999E-2</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="22" spans="1:4" ht="15">
       <c r="A22" s="3" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C22" s="45">
         <f>T_DAYS</f>
         <v>365</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
     </row>
   </sheetData>
@@ -2884,251 +2884,251 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="30" customHeight="1">
-      <c r="A1" s="46" t="s">
-        <v>96</v>
-      </c>
-      <c r="B1" s="46"/>
-      <c r="C1" s="46"/>
-      <c r="D1" s="46"/>
-      <c r="E1" s="46"/>
-      <c r="F1" s="46"/>
+      <c r="A1" s="47" t="s">
+        <v>94</v>
+      </c>
+      <c r="B1" s="47"/>
+      <c r="C1" s="47"/>
+      <c r="D1" s="47"/>
+      <c r="E1" s="47"/>
+      <c r="F1" s="47"/>
     </row>
     <row r="2" spans="1:6" ht="30" customHeight="1">
-      <c r="A2" s="46"/>
-      <c r="B2" s="46"/>
-      <c r="C2" s="46"/>
-      <c r="D2" s="46"/>
-      <c r="E2" s="46"/>
-      <c r="F2" s="46"/>
+      <c r="A2" s="47"/>
+      <c r="B2" s="47"/>
+      <c r="C2" s="47"/>
+      <c r="D2" s="47"/>
+      <c r="E2" s="47"/>
+      <c r="F2" s="47"/>
     </row>
     <row r="3" spans="1:6" ht="15">
-      <c r="A3" s="51" t="s">
-        <v>97</v>
-      </c>
-      <c r="B3" s="51"/>
-      <c r="C3" s="51"/>
-      <c r="D3" s="51"/>
-      <c r="E3" s="51"/>
-      <c r="F3" s="51"/>
+      <c r="A3" s="53" t="s">
+        <v>95</v>
+      </c>
+      <c r="B3" s="53"/>
+      <c r="C3" s="53"/>
+      <c r="D3" s="53"/>
+      <c r="E3" s="53"/>
+      <c r="F3" s="53"/>
     </row>
     <row r="5" spans="1:6" ht="15">
       <c r="A5" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="C5" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="D5" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="E5" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="D5" s="1" t="s">
+      <c r="F5" s="1" t="s">
         <v>101</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>102</v>
-      </c>
-      <c r="F5" s="1" t="s">
-        <v>103</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="15">
       <c r="A6" s="2" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D6" s="16">
         <v>12500000</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="F6" s="12" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="15">
       <c r="A7" s="3" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="D7" s="17">
-        <v>1.08</v>
+        <v>1.1535</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>17</v>
+        <v>243</v>
       </c>
       <c r="F7" s="13" t="s">
-        <v>110</v>
+        <v>245</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="15">
       <c r="A8" s="3" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="D8" s="17">
-        <v>1.091</v>
+        <v>1.1706810000000001</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>112</v>
+        <v>246</v>
       </c>
       <c r="F8" s="13" t="s">
-        <v>113</v>
+        <v>247</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="15">
       <c r="A9" s="3" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="D9" s="18">
-        <v>4.4999999999999998E-2</v>
+        <v>4.0599999999999997E-2</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>17</v>
+        <v>243</v>
       </c>
       <c r="F9" s="13" t="s">
-        <v>116</v>
+        <v>248</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="15">
       <c r="A10" s="3" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="D10" s="18">
-        <v>3.4601911027962513E-2</v>
+        <v>2.5529E-2</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>118</v>
+        <v>243</v>
       </c>
       <c r="F10" s="13" t="s">
-        <v>119</v>
+        <v>249</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="15">
       <c r="A11" s="3" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>120</v>
+        <v>113</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="D11" s="17">
-        <v>1.07</v>
+        <v>1.1535</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>17</v>
+        <v>250</v>
       </c>
       <c r="F11" s="13" t="s">
-        <v>121</v>
+        <v>251</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="15">
       <c r="A12" s="3" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>122</v>
+        <v>114</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="D12" s="17">
-        <v>1.1100000000000001</v>
+        <v>1.1535</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>17</v>
+        <v>250</v>
       </c>
       <c r="F12" s="13" t="s">
-        <v>123</v>
+        <v>251</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="15">
       <c r="A13" s="3" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>124</v>
+        <v>115</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="D13" s="17">
         <v>1.7000000000000001E-2</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="F13" s="13" t="s">
-        <v>125</v>
+        <v>116</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="15">
       <c r="A14" s="3" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>126</v>
+        <v>117</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="D14" s="17">
         <v>2.1999999999999999E-2</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="F14" s="13" t="s">
-        <v>125</v>
+        <v>116</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="15">
       <c r="A15" s="3" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>127</v>
+        <v>118</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>128</v>
+        <v>119</v>
       </c>
       <c r="D15" s="19">
         <v>365</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="F15" s="13" t="s">
-        <v>129</v>
+        <v>120</v>
       </c>
     </row>
   </sheetData>
@@ -3151,75 +3151,75 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="30" customHeight="1">
-      <c r="A1" s="46" t="s">
-        <v>130</v>
-      </c>
-      <c r="B1" s="46"/>
-      <c r="C1" s="46"/>
-      <c r="D1" s="46"/>
-      <c r="E1" s="46"/>
+      <c r="A1" s="47" t="s">
+        <v>121</v>
+      </c>
+      <c r="B1" s="47"/>
+      <c r="C1" s="47"/>
+      <c r="D1" s="47"/>
+      <c r="E1" s="47"/>
     </row>
     <row r="2" spans="1:5" ht="30" customHeight="1">
-      <c r="A2" s="46"/>
-      <c r="B2" s="46"/>
-      <c r="C2" s="46"/>
-      <c r="D2" s="46"/>
-      <c r="E2" s="46"/>
+      <c r="A2" s="47"/>
+      <c r="B2" s="47"/>
+      <c r="C2" s="47"/>
+      <c r="D2" s="47"/>
+      <c r="E2" s="47"/>
     </row>
     <row r="4" spans="1:5" ht="21.95" customHeight="1">
-      <c r="A4" s="47" t="s">
-        <v>131</v>
-      </c>
-      <c r="B4" s="48"/>
-      <c r="C4" s="48"/>
-      <c r="D4" s="48"/>
-      <c r="E4" s="49"/>
+      <c r="A4" s="49" t="s">
+        <v>122</v>
+      </c>
+      <c r="B4" s="50"/>
+      <c r="C4" s="50"/>
+      <c r="D4" s="50"/>
+      <c r="E4" s="51"/>
     </row>
     <row r="5" spans="1:5" ht="15">
       <c r="A5" s="1" t="s">
-        <v>132</v>
+        <v>123</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>133</v>
+        <v>124</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="15">
       <c r="A6" s="2" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B6" s="23">
         <f>FC_AMT</f>
         <v>12500000</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="15">
       <c r="A7" s="3" t="s">
-        <v>134</v>
+        <v>125</v>
       </c>
       <c r="B7" s="24">
         <f>F0_in</f>
-        <v>1.091</v>
+        <v>1.1706810000000001</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="15">
       <c r="A8" s="3" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="B8" s="25">
         <f>T_DAYS</f>
         <v>365</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>128</v>
+        <v>119</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="15">
@@ -3229,50 +3229,50 @@
     </row>
     <row r="10" spans="1:5" ht="15">
       <c r="A10" s="3" t="s">
-        <v>135</v>
+        <v>126</v>
       </c>
       <c r="B10" s="26">
         <f>FC_AMT*F0_in</f>
-        <v>13637500</v>
+        <v>14633512.500000002</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="15">
       <c r="A11" s="3" t="s">
-        <v>136</v>
+        <v>127</v>
       </c>
       <c r="B11" s="27">
         <f>B10/FC_AMT</f>
-        <v>1.091</v>
+        <v>1.1706810000000001</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
     </row>
     <row r="13" spans="1:5">
-      <c r="A13" s="52" t="s">
-        <v>137</v>
-      </c>
-      <c r="B13" s="52"/>
-      <c r="C13" s="52"/>
-      <c r="D13" s="52"/>
-      <c r="E13" s="52"/>
+      <c r="A13" s="54" t="s">
+        <v>128</v>
+      </c>
+      <c r="B13" s="54"/>
+      <c r="C13" s="54"/>
+      <c r="D13" s="54"/>
+      <c r="E13" s="54"/>
     </row>
     <row r="14" spans="1:5">
-      <c r="A14" s="52"/>
-      <c r="B14" s="52"/>
-      <c r="C14" s="52"/>
-      <c r="D14" s="52"/>
-      <c r="E14" s="52"/>
+      <c r="A14" s="54"/>
+      <c r="B14" s="54"/>
+      <c r="C14" s="54"/>
+      <c r="D14" s="54"/>
+      <c r="E14" s="54"/>
     </row>
     <row r="15" spans="1:5">
-      <c r="A15" s="52"/>
-      <c r="B15" s="52"/>
-      <c r="C15" s="52"/>
-      <c r="D15" s="52"/>
-      <c r="E15" s="52"/>
+      <c r="A15" s="54"/>
+      <c r="B15" s="54"/>
+      <c r="C15" s="54"/>
+      <c r="D15" s="54"/>
+      <c r="E15" s="54"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -3297,105 +3297,105 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="30" customHeight="1">
-      <c r="A1" s="46" t="s">
-        <v>138</v>
-      </c>
-      <c r="B1" s="46"/>
-      <c r="C1" s="46"/>
-      <c r="D1" s="46"/>
-      <c r="E1" s="46"/>
-      <c r="F1" s="46"/>
+      <c r="A1" s="47" t="s">
+        <v>129</v>
+      </c>
+      <c r="B1" s="47"/>
+      <c r="C1" s="47"/>
+      <c r="D1" s="47"/>
+      <c r="E1" s="47"/>
+      <c r="F1" s="47"/>
     </row>
     <row r="2" spans="1:6" ht="30" customHeight="1">
-      <c r="A2" s="46"/>
-      <c r="B2" s="46"/>
-      <c r="C2" s="46"/>
-      <c r="D2" s="46"/>
-      <c r="E2" s="46"/>
-      <c r="F2" s="46"/>
+      <c r="A2" s="47"/>
+      <c r="B2" s="47"/>
+      <c r="C2" s="47"/>
+      <c r="D2" s="47"/>
+      <c r="E2" s="47"/>
+      <c r="F2" s="47"/>
     </row>
     <row r="4" spans="1:6" ht="21.95" customHeight="1">
-      <c r="A4" s="47" t="s">
-        <v>139</v>
-      </c>
-      <c r="B4" s="48"/>
-      <c r="C4" s="48"/>
-      <c r="D4" s="48"/>
-      <c r="E4" s="48"/>
-      <c r="F4" s="49"/>
+      <c r="A4" s="49" t="s">
+        <v>130</v>
+      </c>
+      <c r="B4" s="50"/>
+      <c r="C4" s="50"/>
+      <c r="D4" s="50"/>
+      <c r="E4" s="50"/>
+      <c r="F4" s="51"/>
     </row>
     <row r="5" spans="1:6" ht="15">
       <c r="A5" s="1" t="s">
-        <v>140</v>
+        <v>131</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>141</v>
+        <v>132</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>133</v>
+        <v>124</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="15">
       <c r="A6" s="2" t="s">
-        <v>142</v>
+        <v>133</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>143</v>
+        <v>134</v>
       </c>
       <c r="C6" s="28">
         <f>T_DAYS/360</f>
         <v>1.0138888888888888</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>144</v>
+        <v>135</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="15">
       <c r="A7" s="3" t="s">
-        <v>145</v>
+        <v>136</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>146</v>
+        <v>137</v>
       </c>
       <c r="C7" s="29">
         <f>FC_AMT/(1+R_FC*T_DAYS/360)</f>
-        <v>12076332.160014166</v>
+        <v>12184618.578860009</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="15">
       <c r="A8" s="3" t="s">
-        <v>147</v>
+        <v>138</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>148</v>
+        <v>139</v>
       </c>
       <c r="C8" s="30">
         <f>C7*S0_in</f>
-        <v>13042438.732815299</v>
+        <v>14054957.53071502</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="15">
       <c r="A9" s="3" t="s">
-        <v>149</v>
+        <v>140</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>150</v>
+        <v>141</v>
       </c>
       <c r="C9" s="26">
         <f>C8*(1+R_USD*T_DAYS/360)</f>
-        <v>13637499.999999998</v>
+        <v>14633514.240847424</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="15">
@@ -3406,89 +3406,89 @@
     </row>
     <row r="11" spans="1:6" ht="15">
       <c r="A11" s="3" t="s">
-        <v>151</v>
+        <v>142</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>152</v>
+        <v>143</v>
       </c>
       <c r="C11" s="24">
         <f>S0_in*(1+R_USD*T_DAYS/360)/(1+R_FC*T_DAYS/360)</f>
-        <v>1.0909999999999997</v>
+        <v>1.170681139267794</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="15">
       <c r="A12" s="3" t="s">
-        <v>153</v>
+        <v>144</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C12" s="24">
         <f>F0_in</f>
-        <v>1.091</v>
+        <v>1.1706810000000001</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="15">
       <c r="A13" s="3" t="s">
-        <v>154</v>
+        <v>145</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>155</v>
+        <v>146</v>
       </c>
       <c r="C13" s="24">
         <f>C11-C12</f>
-        <v>0</v>
+        <v>1.3926779396378208E-7</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="15">
       <c r="A14" s="3" t="s">
-        <v>136</v>
+        <v>127</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>156</v>
+        <v>147</v>
       </c>
       <c r="C14" s="27">
         <f>C9/FC_AMT</f>
-        <v>1.0909999999999997</v>
+        <v>1.1706811392677938</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
     </row>
     <row r="16" spans="1:6">
-      <c r="A16" s="52" t="s">
-        <v>157</v>
-      </c>
-      <c r="B16" s="52"/>
-      <c r="C16" s="52"/>
-      <c r="D16" s="52"/>
-      <c r="E16" s="52"/>
-      <c r="F16" s="52"/>
+      <c r="A16" s="54" t="s">
+        <v>148</v>
+      </c>
+      <c r="B16" s="54"/>
+      <c r="C16" s="54"/>
+      <c r="D16" s="54"/>
+      <c r="E16" s="54"/>
+      <c r="F16" s="54"/>
     </row>
     <row r="17" spans="1:6">
-      <c r="A17" s="52"/>
-      <c r="B17" s="52"/>
-      <c r="C17" s="52"/>
-      <c r="D17" s="52"/>
-      <c r="E17" s="52"/>
-      <c r="F17" s="52"/>
+      <c r="A17" s="54"/>
+      <c r="B17" s="54"/>
+      <c r="C17" s="54"/>
+      <c r="D17" s="54"/>
+      <c r="E17" s="54"/>
+      <c r="F17" s="54"/>
     </row>
     <row r="18" spans="1:6">
-      <c r="A18" s="52"/>
-      <c r="B18" s="52"/>
-      <c r="C18" s="52"/>
-      <c r="D18" s="52"/>
-      <c r="E18" s="52"/>
-      <c r="F18" s="52"/>
+      <c r="A18" s="54"/>
+      <c r="B18" s="54"/>
+      <c r="C18" s="54"/>
+      <c r="D18" s="54"/>
+      <c r="E18" s="54"/>
+      <c r="F18" s="54"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -3512,213 +3512,213 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="30" customHeight="1">
-      <c r="A1" s="46" t="s">
-        <v>158</v>
-      </c>
-      <c r="B1" s="46"/>
-      <c r="C1" s="46"/>
-      <c r="D1" s="46"/>
-      <c r="E1" s="46"/>
-      <c r="F1" s="46"/>
+      <c r="A1" s="47" t="s">
+        <v>149</v>
+      </c>
+      <c r="B1" s="47"/>
+      <c r="C1" s="47"/>
+      <c r="D1" s="47"/>
+      <c r="E1" s="47"/>
+      <c r="F1" s="47"/>
     </row>
     <row r="2" spans="1:6" ht="30" customHeight="1">
-      <c r="A2" s="46"/>
-      <c r="B2" s="46"/>
-      <c r="C2" s="46"/>
-      <c r="D2" s="46"/>
-      <c r="E2" s="46"/>
-      <c r="F2" s="46"/>
+      <c r="A2" s="47"/>
+      <c r="B2" s="47"/>
+      <c r="C2" s="47"/>
+      <c r="D2" s="47"/>
+      <c r="E2" s="47"/>
+      <c r="F2" s="47"/>
     </row>
     <row r="4" spans="1:6" ht="15">
       <c r="A4" s="2" t="s">
-        <v>159</v>
+        <v>150</v>
       </c>
       <c r="B4" s="2"/>
     </row>
     <row r="5" spans="1:6" ht="15">
       <c r="A5" s="3" t="s">
-        <v>160</v>
+        <v>151</v>
       </c>
       <c r="B5" s="24">
         <f>S0_in</f>
-        <v>1.08</v>
+        <v>1.1535</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="21.95" customHeight="1">
-      <c r="A7" s="47" t="s">
-        <v>161</v>
-      </c>
-      <c r="B7" s="48"/>
-      <c r="C7" s="48"/>
-      <c r="D7" s="48"/>
-      <c r="E7" s="48"/>
-      <c r="F7" s="49"/>
+      <c r="A7" s="49" t="s">
+        <v>152</v>
+      </c>
+      <c r="B7" s="50"/>
+      <c r="C7" s="50"/>
+      <c r="D7" s="50"/>
+      <c r="E7" s="50"/>
+      <c r="F7" s="51"/>
     </row>
     <row r="8" spans="1:6" ht="15">
       <c r="A8" s="1" t="s">
-        <v>132</v>
+        <v>123</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>133</v>
+        <v>124</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="15">
       <c r="A9" s="2" t="s">
-        <v>162</v>
+        <v>153</v>
       </c>
       <c r="B9" s="28">
         <f>MAX(B5,K_PUT)</f>
-        <v>1.08</v>
+        <v>1.1535</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="15">
       <c r="A10" s="3" t="s">
-        <v>163</v>
+        <v>154</v>
       </c>
       <c r="B10" s="24">
         <f>MAX(K_PUT-B5,0)</f>
         <v>0</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="15">
       <c r="A11" s="3" t="s">
-        <v>164</v>
+        <v>155</v>
       </c>
       <c r="B11" s="30">
         <f>FC_AMT*PREM_PUT</f>
         <v>212500.00000000003</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="15">
       <c r="A12" s="3" t="s">
-        <v>165</v>
+        <v>156</v>
       </c>
       <c r="B12" s="26">
         <f>FC_AMT*MAX(B5,K_PUT)-FC_AMT*PREM_PUT</f>
-        <v>13287500</v>
+        <v>14206250</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="15">
       <c r="A13" s="3" t="s">
-        <v>136</v>
+        <v>127</v>
       </c>
       <c r="B13" s="27">
         <f>B12/FC_AMT</f>
-        <v>1.0629999999999999</v>
+        <v>1.1365000000000001</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="21.95" customHeight="1">
-      <c r="A15" s="47" t="s">
-        <v>166</v>
-      </c>
-      <c r="B15" s="48"/>
-      <c r="C15" s="48"/>
-      <c r="D15" s="48"/>
-      <c r="E15" s="48"/>
-      <c r="F15" s="49"/>
+      <c r="A15" s="49" t="s">
+        <v>157</v>
+      </c>
+      <c r="B15" s="50"/>
+      <c r="C15" s="50"/>
+      <c r="D15" s="50"/>
+      <c r="E15" s="50"/>
+      <c r="F15" s="51"/>
     </row>
     <row r="16" spans="1:6" ht="15">
       <c r="A16" s="1" t="s">
-        <v>132</v>
+        <v>123</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>133</v>
+        <v>124</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
     </row>
     <row r="17" spans="1:6" ht="15">
       <c r="A17" s="2" t="s">
-        <v>167</v>
+        <v>158</v>
       </c>
       <c r="B17" s="28">
         <f>MAX(B5-K_CALL,0)</f>
         <v>0</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
     </row>
     <row r="18" spans="1:6" ht="15">
       <c r="A18" s="3" t="s">
-        <v>164</v>
+        <v>155</v>
       </c>
       <c r="B18" s="30">
         <f>FC_AMT*PREM_CALL</f>
         <v>275000</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="19" spans="1:6" ht="15">
       <c r="A19" s="3" t="s">
-        <v>168</v>
+        <v>159</v>
       </c>
       <c r="B19" s="26">
         <f>FC_AMT*B5+FC_AMT*MAX(B5-K_CALL,0)-FC_AMT*PREM_CALL</f>
-        <v>13225000</v>
+        <v>14143750</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="20" spans="1:6" ht="15">
       <c r="A20" s="3" t="s">
-        <v>136</v>
+        <v>127</v>
       </c>
       <c r="B20" s="27">
         <f>B19/FC_AMT</f>
-        <v>1.0580000000000001</v>
+        <v>1.1315</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
     </row>
     <row r="22" spans="1:6">
-      <c r="A22" s="52" t="s">
-        <v>169</v>
-      </c>
-      <c r="B22" s="52"/>
-      <c r="C22" s="52"/>
-      <c r="D22" s="52"/>
-      <c r="E22" s="52"/>
-      <c r="F22" s="52"/>
+      <c r="A22" s="54" t="s">
+        <v>160</v>
+      </c>
+      <c r="B22" s="54"/>
+      <c r="C22" s="54"/>
+      <c r="D22" s="54"/>
+      <c r="E22" s="54"/>
+      <c r="F22" s="54"/>
     </row>
     <row r="23" spans="1:6">
-      <c r="A23" s="52"/>
-      <c r="B23" s="52"/>
-      <c r="C23" s="52"/>
-      <c r="D23" s="52"/>
-      <c r="E23" s="52"/>
-      <c r="F23" s="52"/>
+      <c r="A23" s="54"/>
+      <c r="B23" s="54"/>
+      <c r="C23" s="54"/>
+      <c r="D23" s="54"/>
+      <c r="E23" s="54"/>
+      <c r="F23" s="54"/>
     </row>
     <row r="24" spans="1:6">
-      <c r="A24" s="52"/>
-      <c r="B24" s="52"/>
-      <c r="C24" s="52"/>
-      <c r="D24" s="52"/>
-      <c r="E24" s="52"/>
-      <c r="F24" s="52"/>
+      <c r="A24" s="54"/>
+      <c r="B24" s="54"/>
+      <c r="C24" s="54"/>
+      <c r="D24" s="54"/>
+      <c r="E24" s="54"/>
+      <c r="F24" s="54"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -3743,80 +3743,80 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="30" customHeight="1">
-      <c r="A1" s="46" t="s">
-        <v>170</v>
-      </c>
-      <c r="B1" s="46"/>
-      <c r="C1" s="46"/>
-      <c r="D1" s="46"/>
-      <c r="E1" s="46"/>
-      <c r="F1" s="46"/>
-      <c r="G1" s="46"/>
-      <c r="H1" s="46"/>
-      <c r="I1" s="46"/>
-      <c r="J1" s="46"/>
-      <c r="K1" s="46"/>
-      <c r="L1" s="46"/>
-      <c r="M1" s="46"/>
-      <c r="N1" s="46"/>
-      <c r="O1" s="46"/>
-      <c r="P1" s="46"/>
-      <c r="Q1" s="46"/>
+      <c r="A1" s="47" t="s">
+        <v>161</v>
+      </c>
+      <c r="B1" s="47"/>
+      <c r="C1" s="47"/>
+      <c r="D1" s="47"/>
+      <c r="E1" s="47"/>
+      <c r="F1" s="47"/>
+      <c r="G1" s="47"/>
+      <c r="H1" s="47"/>
+      <c r="I1" s="47"/>
+      <c r="J1" s="47"/>
+      <c r="K1" s="47"/>
+      <c r="L1" s="47"/>
+      <c r="M1" s="47"/>
+      <c r="N1" s="47"/>
+      <c r="O1" s="47"/>
+      <c r="P1" s="47"/>
+      <c r="Q1" s="47"/>
     </row>
     <row r="2" spans="1:17" ht="30" customHeight="1">
-      <c r="A2" s="46"/>
-      <c r="B2" s="46"/>
-      <c r="C2" s="46"/>
-      <c r="D2" s="46"/>
-      <c r="E2" s="46"/>
-      <c r="F2" s="46"/>
-      <c r="G2" s="46"/>
-      <c r="H2" s="46"/>
-      <c r="I2" s="46"/>
-      <c r="J2" s="46"/>
-      <c r="K2" s="46"/>
-      <c r="L2" s="46"/>
-      <c r="M2" s="46"/>
-      <c r="N2" s="46"/>
-      <c r="O2" s="46"/>
-      <c r="P2" s="46"/>
-      <c r="Q2" s="46"/>
+      <c r="A2" s="47"/>
+      <c r="B2" s="47"/>
+      <c r="C2" s="47"/>
+      <c r="D2" s="47"/>
+      <c r="E2" s="47"/>
+      <c r="F2" s="47"/>
+      <c r="G2" s="47"/>
+      <c r="H2" s="47"/>
+      <c r="I2" s="47"/>
+      <c r="J2" s="47"/>
+      <c r="K2" s="47"/>
+      <c r="L2" s="47"/>
+      <c r="M2" s="47"/>
+      <c r="N2" s="47"/>
+      <c r="O2" s="47"/>
+      <c r="P2" s="47"/>
+      <c r="Q2" s="47"/>
     </row>
     <row r="3" spans="1:17" ht="15.75">
-      <c r="A3" s="53" t="s">
-        <v>171</v>
-      </c>
-      <c r="B3" s="53"/>
-      <c r="C3" s="53"/>
-      <c r="D3" s="53"/>
-      <c r="E3" s="53"/>
-      <c r="F3" s="53"/>
-      <c r="G3" s="53"/>
+      <c r="A3" s="48" t="s">
+        <v>162</v>
+      </c>
+      <c r="B3" s="48"/>
+      <c r="C3" s="48"/>
+      <c r="D3" s="48"/>
+      <c r="E3" s="48"/>
+      <c r="F3" s="48"/>
+      <c r="G3" s="48"/>
     </row>
     <row r="5" spans="1:17" ht="15">
       <c r="A5" s="1" t="s">
-        <v>172</v>
+        <v>163</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>173</v>
+        <v>164</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H5" s="35" t="s">
-        <v>174</v>
+        <v>165</v>
       </c>
     </row>
     <row r="6" spans="1:17" ht="15">
@@ -3826,27 +3826,27 @@
       </c>
       <c r="B6" s="28">
         <f t="shared" ref="B6:B16" si="0">A6*S0_in</f>
-        <v>1.026</v>
+        <v>1.0958249999999998</v>
       </c>
       <c r="C6" s="34">
         <f t="shared" ref="C6:C16" si="1">FC_AMT*B6</f>
-        <v>12825000</v>
+        <v>13697812.499999998</v>
       </c>
       <c r="D6" s="34">
         <f>'Forward Hedge'!$B$10</f>
-        <v>13637500</v>
+        <v>14633512.500000002</v>
       </c>
       <c r="E6" s="34">
         <f>'Money Market'!$C$9</f>
-        <v>13637499.999999998</v>
+        <v>14633514.240847424</v>
       </c>
       <c r="F6" s="34">
         <f t="shared" ref="F6:F16" si="2">FC_AMT*MAX(B6,K_PUT)-FC_AMT*PREM_PUT</f>
-        <v>13162500</v>
+        <v>14206250</v>
       </c>
       <c r="G6" s="34">
         <f t="shared" ref="G6:G16" si="3">FC_AMT*B6+FC_AMT*MAX(B6-K_CALL,0)-FC_AMT*PREM_CALL</f>
-        <v>12550000</v>
+        <v>13422812.499999998</v>
       </c>
       <c r="H6" s="35" t="str">
         <f t="shared" ref="H6:H16" si="4">TEXT(A6,"0%")</f>
@@ -3860,27 +3860,27 @@
       </c>
       <c r="B7" s="24">
         <f t="shared" si="0"/>
-        <v>1.0367999999999999</v>
+        <v>1.1073599999999999</v>
       </c>
       <c r="C7" s="26">
         <f t="shared" si="1"/>
-        <v>12960000</v>
+        <v>13841999.999999998</v>
       </c>
       <c r="D7" s="26">
         <f>'Forward Hedge'!$B$10</f>
-        <v>13637500</v>
+        <v>14633512.500000002</v>
       </c>
       <c r="E7" s="26">
         <f>'Money Market'!$C$9</f>
-        <v>13637499.999999998</v>
+        <v>14633514.240847424</v>
       </c>
       <c r="F7" s="26">
         <f t="shared" si="2"/>
-        <v>13162500</v>
+        <v>14206250</v>
       </c>
       <c r="G7" s="26">
         <f t="shared" si="3"/>
-        <v>12685000</v>
+        <v>13566999.999999998</v>
       </c>
       <c r="H7" s="35" t="str">
         <f t="shared" si="4"/>
@@ -3894,27 +3894,27 @@
       </c>
       <c r="B8" s="24">
         <f t="shared" si="0"/>
-        <v>1.0476000000000001</v>
+        <v>1.118895</v>
       </c>
       <c r="C8" s="26">
         <f t="shared" si="1"/>
-        <v>13095000.000000002</v>
+        <v>13986187.5</v>
       </c>
       <c r="D8" s="26">
         <f>'Forward Hedge'!$B$10</f>
-        <v>13637500</v>
+        <v>14633512.500000002</v>
       </c>
       <c r="E8" s="26">
         <f>'Money Market'!$C$9</f>
-        <v>13637499.999999998</v>
+        <v>14633514.240847424</v>
       </c>
       <c r="F8" s="26">
         <f t="shared" si="2"/>
-        <v>13162500</v>
+        <v>14206250</v>
       </c>
       <c r="G8" s="26">
         <f t="shared" si="3"/>
-        <v>12820000.000000002</v>
+        <v>13711187.5</v>
       </c>
       <c r="H8" s="35" t="str">
         <f t="shared" si="4"/>
@@ -3928,27 +3928,27 @@
       </c>
       <c r="B9" s="24">
         <f t="shared" si="0"/>
-        <v>1.0584</v>
+        <v>1.13043</v>
       </c>
       <c r="C9" s="26">
         <f t="shared" si="1"/>
-        <v>13230000</v>
+        <v>14130375</v>
       </c>
       <c r="D9" s="26">
         <f>'Forward Hedge'!$B$10</f>
-        <v>13637500</v>
+        <v>14633512.500000002</v>
       </c>
       <c r="E9" s="26">
         <f>'Money Market'!$C$9</f>
-        <v>13637499.999999998</v>
+        <v>14633514.240847424</v>
       </c>
       <c r="F9" s="26">
         <f t="shared" si="2"/>
-        <v>13162500</v>
+        <v>14206250</v>
       </c>
       <c r="G9" s="26">
         <f t="shared" si="3"/>
-        <v>12955000</v>
+        <v>13855375</v>
       </c>
       <c r="H9" s="35" t="str">
         <f t="shared" si="4"/>
@@ -3962,27 +3962,27 @@
       </c>
       <c r="B10" s="24">
         <f t="shared" si="0"/>
-        <v>1.0692000000000002</v>
+        <v>1.1419649999999999</v>
       </c>
       <c r="C10" s="26">
         <f t="shared" si="1"/>
-        <v>13365000.000000002</v>
+        <v>14274562.499999998</v>
       </c>
       <c r="D10" s="26">
         <f>'Forward Hedge'!$B$10</f>
-        <v>13637500</v>
+        <v>14633512.500000002</v>
       </c>
       <c r="E10" s="26">
         <f>'Money Market'!$C$9</f>
-        <v>13637499.999999998</v>
+        <v>14633514.240847424</v>
       </c>
       <c r="F10" s="26">
         <f t="shared" si="2"/>
-        <v>13162500</v>
+        <v>14206250</v>
       </c>
       <c r="G10" s="26">
         <f t="shared" si="3"/>
-        <v>13090000.000000002</v>
+        <v>13999562.499999998</v>
       </c>
       <c r="H10" s="35" t="str">
         <f t="shared" si="4"/>
@@ -3996,27 +3996,27 @@
       </c>
       <c r="B11" s="24">
         <f t="shared" si="0"/>
-        <v>1.08</v>
+        <v>1.1535</v>
       </c>
       <c r="C11" s="26">
         <f t="shared" si="1"/>
-        <v>13500000</v>
+        <v>14418750</v>
       </c>
       <c r="D11" s="26">
         <f>'Forward Hedge'!$B$10</f>
-        <v>13637500</v>
+        <v>14633512.500000002</v>
       </c>
       <c r="E11" s="26">
         <f>'Money Market'!$C$9</f>
-        <v>13637499.999999998</v>
+        <v>14633514.240847424</v>
       </c>
       <c r="F11" s="26">
         <f t="shared" si="2"/>
-        <v>13287500</v>
+        <v>14206250</v>
       </c>
       <c r="G11" s="26">
         <f t="shared" si="3"/>
-        <v>13225000</v>
+        <v>14143750</v>
       </c>
       <c r="H11" s="35" t="str">
         <f t="shared" si="4"/>
@@ -4030,27 +4030,27 @@
       </c>
       <c r="B12" s="24">
         <f t="shared" si="0"/>
-        <v>1.0908</v>
+        <v>1.165035</v>
       </c>
       <c r="C12" s="26">
         <f t="shared" si="1"/>
-        <v>13635000</v>
+        <v>14562937.5</v>
       </c>
       <c r="D12" s="26">
         <f>'Forward Hedge'!$B$10</f>
-        <v>13637500</v>
+        <v>14633512.500000002</v>
       </c>
       <c r="E12" s="26">
         <f>'Money Market'!$C$9</f>
-        <v>13637499.999999998</v>
+        <v>14633514.240847424</v>
       </c>
       <c r="F12" s="26">
         <f t="shared" si="2"/>
-        <v>13422500</v>
+        <v>14350437.5</v>
       </c>
       <c r="G12" s="26">
         <f t="shared" si="3"/>
-        <v>13360000</v>
+        <v>14432125</v>
       </c>
       <c r="H12" s="35" t="str">
         <f t="shared" si="4"/>
@@ -4064,27 +4064,27 @@
       </c>
       <c r="B13" s="24">
         <f t="shared" si="0"/>
-        <v>1.1016000000000001</v>
+        <v>1.1765699999999999</v>
       </c>
       <c r="C13" s="26">
         <f t="shared" si="1"/>
-        <v>13770000.000000002</v>
+        <v>14707124.999999998</v>
       </c>
       <c r="D13" s="26">
         <f>'Forward Hedge'!$B$10</f>
-        <v>13637500</v>
+        <v>14633512.500000002</v>
       </c>
       <c r="E13" s="26">
         <f>'Money Market'!$C$9</f>
-        <v>13637499.999999998</v>
+        <v>14633514.240847424</v>
       </c>
       <c r="F13" s="26">
         <f t="shared" si="2"/>
-        <v>13557500.000000002</v>
+        <v>14494624.999999998</v>
       </c>
       <c r="G13" s="26">
         <f t="shared" si="3"/>
-        <v>13495000.000000002</v>
+        <v>14720499.999999996</v>
       </c>
       <c r="H13" s="35" t="str">
         <f t="shared" si="4"/>
@@ -4098,27 +4098,27 @@
       </c>
       <c r="B14" s="24">
         <f t="shared" si="0"/>
-        <v>1.1124000000000001</v>
+        <v>1.188105</v>
       </c>
       <c r="C14" s="26">
         <f t="shared" si="1"/>
-        <v>13905000</v>
+        <v>14851312.5</v>
       </c>
       <c r="D14" s="26">
         <f>'Forward Hedge'!$B$10</f>
-        <v>13637500</v>
+        <v>14633512.500000002</v>
       </c>
       <c r="E14" s="26">
         <f>'Money Market'!$C$9</f>
-        <v>13637499.999999998</v>
+        <v>14633514.240847424</v>
       </c>
       <c r="F14" s="26">
         <f t="shared" si="2"/>
-        <v>13692500</v>
+        <v>14638812.5</v>
       </c>
       <c r="G14" s="26">
         <f t="shared" si="3"/>
-        <v>13660000</v>
+        <v>15008875</v>
       </c>
       <c r="H14" s="35" t="str">
         <f t="shared" si="4"/>
@@ -4132,27 +4132,27 @@
       </c>
       <c r="B15" s="24">
         <f t="shared" si="0"/>
-        <v>1.1232000000000002</v>
+        <v>1.19964</v>
       </c>
       <c r="C15" s="26">
         <f t="shared" si="1"/>
-        <v>14040000.000000002</v>
+        <v>14995500</v>
       </c>
       <c r="D15" s="26">
         <f>'Forward Hedge'!$B$10</f>
-        <v>13637500</v>
+        <v>14633512.500000002</v>
       </c>
       <c r="E15" s="26">
         <f>'Money Market'!$C$9</f>
-        <v>13637499.999999998</v>
+        <v>14633514.240847424</v>
       </c>
       <c r="F15" s="26">
         <f t="shared" si="2"/>
-        <v>13827500.000000002</v>
+        <v>14783000</v>
       </c>
       <c r="G15" s="26">
         <f t="shared" si="3"/>
-        <v>13930000.000000004</v>
+        <v>15297250</v>
       </c>
       <c r="H15" s="35" t="str">
         <f t="shared" si="4"/>
@@ -4166,27 +4166,27 @@
       </c>
       <c r="B16" s="24">
         <f t="shared" si="0"/>
-        <v>1.1340000000000001</v>
+        <v>1.2111750000000001</v>
       </c>
       <c r="C16" s="26">
         <f t="shared" si="1"/>
-        <v>14175000.000000002</v>
+        <v>15139687.500000002</v>
       </c>
       <c r="D16" s="26">
         <f>'Forward Hedge'!$B$10</f>
-        <v>13637500</v>
+        <v>14633512.500000002</v>
       </c>
       <c r="E16" s="26">
         <f>'Money Market'!$C$9</f>
-        <v>13637499.999999998</v>
+        <v>14633514.240847424</v>
       </c>
       <c r="F16" s="26">
         <f t="shared" si="2"/>
-        <v>13962500.000000002</v>
+        <v>14927187.500000002</v>
       </c>
       <c r="G16" s="26">
         <f t="shared" si="3"/>
-        <v>14200000.000000002</v>
+        <v>15585625.000000004</v>
       </c>
       <c r="H16" s="35" t="str">
         <f t="shared" si="4"/>
@@ -4215,24 +4215,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="30" customHeight="1">
-      <c r="A1" s="46" t="s">
-        <v>175</v>
-      </c>
-      <c r="B1" s="46"/>
-      <c r="C1" s="46"/>
-      <c r="D1" s="46"/>
-      <c r="E1" s="46"/>
-      <c r="F1" s="46"/>
-      <c r="G1" s="46"/>
+      <c r="A1" s="47" t="s">
+        <v>166</v>
+      </c>
+      <c r="B1" s="47"/>
+      <c r="C1" s="47"/>
+      <c r="D1" s="47"/>
+      <c r="E1" s="47"/>
+      <c r="F1" s="47"/>
+      <c r="G1" s="47"/>
     </row>
     <row r="2" spans="1:7" ht="30" customHeight="1">
-      <c r="A2" s="46"/>
-      <c r="B2" s="46"/>
-      <c r="C2" s="46"/>
-      <c r="D2" s="46"/>
-      <c r="E2" s="46"/>
-      <c r="F2" s="46"/>
-      <c r="G2" s="46"/>
+      <c r="A2" s="47"/>
+      <c r="B2" s="47"/>
+      <c r="C2" s="47"/>
+      <c r="D2" s="47"/>
+      <c r="E2" s="47"/>
+      <c r="F2" s="47"/>
+      <c r="G2" s="47"/>
     </row>
     <row r="3" spans="1:7" ht="18">
       <c r="A3" s="36" t="s">
@@ -4245,30 +4245,30 @@
     </row>
     <row r="5" spans="1:7" ht="15">
       <c r="A5" s="1" t="s">
-        <v>176</v>
+        <v>167</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>178</v>
+        <v>169</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>179</v>
+        <v>170</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>180</v>
+        <v>171</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>181</v>
+        <v>172</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="15">
       <c r="A6" s="2" t="s">
-        <v>182</v>
+        <v>173</v>
       </c>
       <c r="B6" s="38">
         <f>COUNT(FC_AMT,S0_in,F0_in,R_USD,R_FC,K_PUT,K_CALL,PREM_PUT,PREM_CALL,T_DAYS)</f>
@@ -4291,12 +4291,12 @@
         <v>PASS</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>183</v>
+        <v>174</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="15">
       <c r="A7" s="3" t="s">
-        <v>184</v>
+        <v>175</v>
       </c>
       <c r="B7" s="39">
         <f>MIN(FC_AMT,S0_in,F0_in,K_PUT,K_CALL,T_DAYS,PREM_PUT,PREM_CALL)</f>
@@ -4319,20 +4319,20 @@
         <v>PASS</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>183</v>
+        <v>174</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="15">
       <c r="A8" s="3" t="s">
-        <v>185</v>
+        <v>176</v>
       </c>
       <c r="B8" s="30">
         <f>'Forward Hedge'!B10</f>
-        <v>13637500</v>
+        <v>14633512.500000002</v>
       </c>
       <c r="C8" s="30">
         <f>FC_AMT*F0_in</f>
-        <v>13637500</v>
+        <v>14633512.500000002</v>
       </c>
       <c r="D8" s="30">
         <f t="shared" si="0"/>
@@ -4347,76 +4347,76 @@
         <v>PASS</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>186</v>
+        <v>177</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="15">
       <c r="A9" s="3" t="s">
-        <v>187</v>
+        <v>178</v>
       </c>
       <c r="B9" s="24">
         <f>'Money Market'!C11</f>
-        <v>1.0909999999999997</v>
+        <v>1.170681139267794</v>
       </c>
       <c r="C9" s="24">
         <f>F0_in</f>
-        <v>1.091</v>
+        <v>1.1706810000000001</v>
       </c>
       <c r="D9" s="24">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1.3926779396378208E-7</v>
       </c>
       <c r="E9" s="24">
         <f>ABS(C9)*'Notes &amp; Assumptions'!B15</f>
-        <v>5.4549999999999998E-3</v>
+        <v>5.8534050000000008E-3</v>
       </c>
       <c r="F9" s="22" t="str">
         <f>IF(ABS(D9)&lt;=E9,"PASS","FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>188</v>
+        <v>179</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="15">
       <c r="A10" s="3" t="s">
-        <v>189</v>
+        <v>180</v>
       </c>
       <c r="B10" s="30">
         <f>'Money Market'!C9</f>
-        <v>13637499.999999998</v>
+        <v>14633514.240847424</v>
       </c>
       <c r="C10" s="30">
         <f>'Forward Hedge'!B10</f>
-        <v>13637500</v>
+        <v>14633512.500000002</v>
       </c>
       <c r="D10" s="30">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1.7408474218100309</v>
       </c>
       <c r="E10" s="30">
         <f>ABS(C10)*'Notes &amp; Assumptions'!B15</f>
-        <v>68187.5</v>
+        <v>73167.562500000015</v>
       </c>
       <c r="F10" s="22" t="str">
         <f>IF(ABS(D10)&lt;=E10,"PASS","FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>190</v>
+        <v>181</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="15">
       <c r="A11" s="3" t="s">
-        <v>191</v>
+        <v>182</v>
       </c>
       <c r="B11" s="30">
         <f>MIN(Sensitivity!F6:F16)</f>
-        <v>13162500</v>
+        <v>14206250</v>
       </c>
       <c r="C11" s="30">
         <f>FC_AMT*K_PUT-FC_AMT*PREM_PUT</f>
-        <v>13162500</v>
+        <v>14206250</v>
       </c>
       <c r="D11" s="30">
         <f t="shared" si="0"/>
@@ -4431,12 +4431,12 @@
         <v>PASS</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="15">
       <c r="A12" s="3" t="s">
-        <v>193</v>
+        <v>184</v>
       </c>
       <c r="B12" s="25">
         <f>COUNT(Sensitivity!B6:B16)</f>
@@ -4459,12 +4459,12 @@
         <v>PASS</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>194</v>
+        <v>185</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="15">
       <c r="A13" s="3" t="s">
-        <v>195</v>
+        <v>186</v>
       </c>
       <c r="B13" s="39">
         <f>MAX(ABS(Sensitivity!B6-S0_in*'Notes &amp; Assumptions'!B12),ABS(Sensitivity!B16-S0_in*('Notes &amp; Assumptions'!B12+('Notes &amp; Assumptions'!B14-1)*'Notes &amp; Assumptions'!B13)))</f>
@@ -4487,7 +4487,7 @@
         <v>PASS</v>
       </c>
       <c r="G13" s="3" t="s">
-        <v>196</v>
+        <v>187</v>
       </c>
     </row>
   </sheetData>
@@ -4520,314 +4520,314 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="30" customHeight="1">
-      <c r="A1" s="46" t="s">
-        <v>197</v>
-      </c>
-      <c r="B1" s="46"/>
-      <c r="C1" s="46"/>
-      <c r="D1" s="46"/>
-      <c r="E1" s="46"/>
-      <c r="F1" s="46"/>
+      <c r="A1" s="47" t="s">
+        <v>188</v>
+      </c>
+      <c r="B1" s="47"/>
+      <c r="C1" s="47"/>
+      <c r="D1" s="47"/>
+      <c r="E1" s="47"/>
+      <c r="F1" s="47"/>
     </row>
     <row r="2" spans="1:6" ht="30" customHeight="1">
-      <c r="A2" s="46"/>
-      <c r="B2" s="46"/>
-      <c r="C2" s="46"/>
-      <c r="D2" s="46"/>
-      <c r="E2" s="46"/>
-      <c r="F2" s="46"/>
+      <c r="A2" s="47"/>
+      <c r="B2" s="47"/>
+      <c r="C2" s="47"/>
+      <c r="D2" s="47"/>
+      <c r="E2" s="47"/>
+      <c r="F2" s="47"/>
     </row>
     <row r="4" spans="1:6" ht="21.95" customHeight="1">
-      <c r="A4" s="47" t="s">
-        <v>198</v>
-      </c>
-      <c r="B4" s="48"/>
-      <c r="C4" s="48"/>
-      <c r="D4" s="48"/>
-      <c r="E4" s="48"/>
-      <c r="F4" s="49"/>
+      <c r="A4" s="49" t="s">
+        <v>189</v>
+      </c>
+      <c r="B4" s="50"/>
+      <c r="C4" s="50"/>
+      <c r="D4" s="50"/>
+      <c r="E4" s="50"/>
+      <c r="F4" s="51"/>
     </row>
     <row r="5" spans="1:6" ht="15">
       <c r="A5" s="1" t="s">
-        <v>199</v>
+        <v>190</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>133</v>
+        <v>124</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>200</v>
+        <v>191</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="15">
       <c r="A6" s="2" t="s">
-        <v>201</v>
+        <v>192</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>202</v>
+        <v>193</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>203</v>
+        <v>194</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="15">
       <c r="A7" s="3" t="s">
-        <v>204</v>
+        <v>195</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>205</v>
+        <v>196</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>206</v>
+        <v>197</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="15">
       <c r="A8" s="3" t="s">
-        <v>207</v>
+        <v>198</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>208</v>
+        <v>199</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>209</v>
+        <v>200</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="15">
       <c r="A9" s="3" t="s">
-        <v>210</v>
+        <v>201</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>211</v>
+        <v>202</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>212</v>
+        <v>203</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="15">
       <c r="A10" s="3" t="s">
-        <v>213</v>
+        <v>204</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>214</v>
+        <v>205</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="15">
       <c r="A11" s="3" t="s">
-        <v>215</v>
+        <v>206</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>216</v>
+        <v>207</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>217</v>
+        <v>208</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="15">
       <c r="A12" s="3" t="s">
-        <v>218</v>
+        <v>209</v>
       </c>
       <c r="B12" s="6">
         <v>0.95</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>219</v>
+        <v>210</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="15">
       <c r="A13" s="3" t="s">
-        <v>220</v>
+        <v>211</v>
       </c>
       <c r="B13" s="6">
         <v>0.01</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>221</v>
+        <v>212</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="15">
       <c r="A14" s="3" t="s">
-        <v>222</v>
+        <v>213</v>
       </c>
       <c r="B14" s="7">
         <v>11</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>223</v>
+        <v>214</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="15">
       <c r="A15" s="3" t="s">
-        <v>224</v>
+        <v>215</v>
       </c>
       <c r="B15" s="6">
         <v>5.0000000000000001E-3</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>225</v>
+        <v>216</v>
       </c>
     </row>
     <row r="16" spans="1:6" ht="15">
       <c r="A16" s="3" t="s">
-        <v>226</v>
+        <v>217</v>
       </c>
       <c r="B16" s="8">
         <v>0.01</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>227</v>
+        <v>218</v>
       </c>
     </row>
     <row r="17" spans="1:6" ht="15">
       <c r="A17" s="3" t="s">
-        <v>228</v>
+        <v>219</v>
       </c>
       <c r="B17" s="7">
         <v>10</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>229</v>
+        <v>220</v>
       </c>
     </row>
     <row r="18" spans="1:6" ht="15">
       <c r="A18" s="3" t="s">
-        <v>230</v>
+        <v>221</v>
       </c>
       <c r="B18" s="7">
         <v>0</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>231</v>
+        <v>222</v>
       </c>
     </row>
     <row r="19" spans="1:6" ht="15">
       <c r="A19" s="3" t="s">
-        <v>232</v>
+        <v>223</v>
       </c>
       <c r="B19" s="9">
         <v>9.9999999999999995E-7</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>233</v>
+        <v>224</v>
       </c>
     </row>
     <row r="21" spans="1:6" ht="21.95" customHeight="1">
-      <c r="A21" s="47" t="s">
-        <v>234</v>
-      </c>
-      <c r="B21" s="48"/>
-      <c r="C21" s="48"/>
-      <c r="D21" s="48"/>
-      <c r="E21" s="48"/>
-      <c r="F21" s="49"/>
+      <c r="A21" s="49" t="s">
+        <v>225</v>
+      </c>
+      <c r="B21" s="50"/>
+      <c r="C21" s="50"/>
+      <c r="D21" s="50"/>
+      <c r="E21" s="50"/>
+      <c r="F21" s="51"/>
     </row>
     <row r="22" spans="1:6" ht="15">
-      <c r="A22" s="57" t="s">
-        <v>235</v>
-      </c>
-      <c r="B22" s="58"/>
-      <c r="C22" s="58"/>
-      <c r="D22" s="58"/>
-      <c r="E22" s="58"/>
-      <c r="F22" s="59"/>
+      <c r="A22" s="58" t="s">
+        <v>226</v>
+      </c>
+      <c r="B22" s="59"/>
+      <c r="C22" s="59"/>
+      <c r="D22" s="59"/>
+      <c r="E22" s="59"/>
+      <c r="F22" s="60"/>
     </row>
     <row r="23" spans="1:6" ht="15">
-      <c r="A23" s="60" t="s">
-        <v>236</v>
-      </c>
-      <c r="B23" s="61"/>
-      <c r="C23" s="61"/>
-      <c r="D23" s="61"/>
-      <c r="E23" s="61"/>
-      <c r="F23" s="62"/>
+      <c r="A23" s="61" t="s">
+        <v>227</v>
+      </c>
+      <c r="B23" s="62"/>
+      <c r="C23" s="62"/>
+      <c r="D23" s="62"/>
+      <c r="E23" s="62"/>
+      <c r="F23" s="63"/>
     </row>
     <row r="24" spans="1:6" ht="15">
-      <c r="A24" s="54" t="s">
-        <v>237</v>
-      </c>
-      <c r="B24" s="55"/>
-      <c r="C24" s="55"/>
-      <c r="D24" s="55"/>
-      <c r="E24" s="55"/>
-      <c r="F24" s="56"/>
+      <c r="A24" s="55" t="s">
+        <v>228</v>
+      </c>
+      <c r="B24" s="56"/>
+      <c r="C24" s="56"/>
+      <c r="D24" s="56"/>
+      <c r="E24" s="56"/>
+      <c r="F24" s="57"/>
     </row>
     <row r="26" spans="1:6" ht="21.95" customHeight="1">
-      <c r="A26" s="47" t="s">
-        <v>238</v>
-      </c>
-      <c r="B26" s="48"/>
-      <c r="C26" s="48"/>
-      <c r="D26" s="48"/>
-      <c r="E26" s="48"/>
-      <c r="F26" s="49"/>
+      <c r="A26" s="49" t="s">
+        <v>229</v>
+      </c>
+      <c r="B26" s="50"/>
+      <c r="C26" s="50"/>
+      <c r="D26" s="50"/>
+      <c r="E26" s="50"/>
+      <c r="F26" s="51"/>
     </row>
     <row r="27" spans="1:6" ht="15">
       <c r="A27" s="1" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>240</v>
+        <v>231</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>241</v>
+        <v>232</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>242</v>
+        <v>233</v>
       </c>
     </row>
     <row r="28" spans="1:6" ht="30">
       <c r="A28" s="2" t="s">
-        <v>243</v>
+        <v>234</v>
       </c>
       <c r="B28" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C28" s="10" t="s">
-        <v>244</v>
+        <v>235</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E28" s="12" t="s">
-        <v>245</v>
+        <v>236</v>
       </c>
     </row>
     <row r="29" spans="1:6" ht="28.5">
       <c r="A29" s="3" t="s">
-        <v>246</v>
+        <v>237</v>
       </c>
       <c r="B29" s="3" t="s">
         <v>12</v>
       </c>
       <c r="C29" s="11" t="s">
-        <v>247</v>
+        <v>238</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E29" s="13" t="s">
-        <v>248</v>
+        <v>239</v>
       </c>
     </row>
     <row r="30" spans="1:6" ht="15">
       <c r="A30" s="3" t="s">
-        <v>249</v>
+        <v>240</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>216</v>
+        <v>207</v>
       </c>
       <c r="C30" s="11" t="s">
-        <v>250</v>
+        <v>241</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E30" s="13" t="s">
-        <v>251</v>
+        <v>242</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Complete Stage 5 validation and hedge recommendation
</commit_message>
<xml_diff>
--- a/models/builds/2026-08-08-Vuong-tech-services-model.xlsx
+++ b/models/builds/2026-08-08-Vuong-tech-services-model.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vuong\OneDrive\Documents\GitHub\Timmy Vuong\models\builds\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/bb7fa6db8e3c4ce1/Documents/GitHub/Timmy Vuong/models/builds/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8753436-C22A-4313-8ADE-BFB3844813CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="13_ncr:1_{A8753436-C22A-4313-8ADE-BFB3844813CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{94CE566A-8C0A-4252-9655-F48E019A75AF}"/>
   <bookViews>
-    <workbookView xWindow="2895" yWindow="375" windowWidth="23820" windowHeight="19890" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="26010" windowHeight="20985" firstSheet="2" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cover" sheetId="1" r:id="rId1"/>
@@ -1252,26 +1252,26 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -2902,14 +2902,14 @@
       <c r="F2" s="47"/>
     </row>
     <row r="3" spans="1:6" ht="15">
-      <c r="A3" s="53" t="s">
+      <c r="A3" s="48" t="s">
         <v>95</v>
       </c>
-      <c r="B3" s="53"/>
-      <c r="C3" s="53"/>
-      <c r="D3" s="53"/>
-      <c r="E3" s="53"/>
-      <c r="F3" s="53"/>
+      <c r="B3" s="48"/>
+      <c r="C3" s="48"/>
+      <c r="D3" s="48"/>
+      <c r="E3" s="48"/>
+      <c r="F3" s="48"/>
     </row>
     <row r="5" spans="1:6" ht="15">
       <c r="A5" s="1" t="s">
@@ -3252,27 +3252,27 @@
       </c>
     </row>
     <row r="13" spans="1:5">
-      <c r="A13" s="54" t="s">
+      <c r="A13" s="53" t="s">
         <v>128</v>
       </c>
-      <c r="B13" s="54"/>
-      <c r="C13" s="54"/>
-      <c r="D13" s="54"/>
-      <c r="E13" s="54"/>
+      <c r="B13" s="53"/>
+      <c r="C13" s="53"/>
+      <c r="D13" s="53"/>
+      <c r="E13" s="53"/>
     </row>
     <row r="14" spans="1:5">
-      <c r="A14" s="54"/>
-      <c r="B14" s="54"/>
-      <c r="C14" s="54"/>
-      <c r="D14" s="54"/>
-      <c r="E14" s="54"/>
+      <c r="A14" s="53"/>
+      <c r="B14" s="53"/>
+      <c r="C14" s="53"/>
+      <c r="D14" s="53"/>
+      <c r="E14" s="53"/>
     </row>
     <row r="15" spans="1:5">
-      <c r="A15" s="54"/>
-      <c r="B15" s="54"/>
-      <c r="C15" s="54"/>
-      <c r="D15" s="54"/>
-      <c r="E15" s="54"/>
+      <c r="A15" s="53"/>
+      <c r="B15" s="53"/>
+      <c r="C15" s="53"/>
+      <c r="D15" s="53"/>
+      <c r="E15" s="53"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -3465,30 +3465,30 @@
       </c>
     </row>
     <row r="16" spans="1:6">
-      <c r="A16" s="54" t="s">
+      <c r="A16" s="53" t="s">
         <v>148</v>
       </c>
-      <c r="B16" s="54"/>
-      <c r="C16" s="54"/>
-      <c r="D16" s="54"/>
-      <c r="E16" s="54"/>
-      <c r="F16" s="54"/>
+      <c r="B16" s="53"/>
+      <c r="C16" s="53"/>
+      <c r="D16" s="53"/>
+      <c r="E16" s="53"/>
+      <c r="F16" s="53"/>
     </row>
     <row r="17" spans="1:6">
-      <c r="A17" s="54"/>
-      <c r="B17" s="54"/>
-      <c r="C17" s="54"/>
-      <c r="D17" s="54"/>
-      <c r="E17" s="54"/>
-      <c r="F17" s="54"/>
+      <c r="A17" s="53"/>
+      <c r="B17" s="53"/>
+      <c r="C17" s="53"/>
+      <c r="D17" s="53"/>
+      <c r="E17" s="53"/>
+      <c r="F17" s="53"/>
     </row>
     <row r="18" spans="1:6">
-      <c r="A18" s="54"/>
-      <c r="B18" s="54"/>
-      <c r="C18" s="54"/>
-      <c r="D18" s="54"/>
-      <c r="E18" s="54"/>
-      <c r="F18" s="54"/>
+      <c r="A18" s="53"/>
+      <c r="B18" s="53"/>
+      <c r="C18" s="53"/>
+      <c r="D18" s="53"/>
+      <c r="E18" s="53"/>
+      <c r="F18" s="53"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -3695,30 +3695,30 @@
       </c>
     </row>
     <row r="22" spans="1:6">
-      <c r="A22" s="54" t="s">
+      <c r="A22" s="53" t="s">
         <v>160</v>
       </c>
-      <c r="B22" s="54"/>
-      <c r="C22" s="54"/>
-      <c r="D22" s="54"/>
-      <c r="E22" s="54"/>
-      <c r="F22" s="54"/>
+      <c r="B22" s="53"/>
+      <c r="C22" s="53"/>
+      <c r="D22" s="53"/>
+      <c r="E22" s="53"/>
+      <c r="F22" s="53"/>
     </row>
     <row r="23" spans="1:6">
-      <c r="A23" s="54"/>
-      <c r="B23" s="54"/>
-      <c r="C23" s="54"/>
-      <c r="D23" s="54"/>
-      <c r="E23" s="54"/>
-      <c r="F23" s="54"/>
+      <c r="A23" s="53"/>
+      <c r="B23" s="53"/>
+      <c r="C23" s="53"/>
+      <c r="D23" s="53"/>
+      <c r="E23" s="53"/>
+      <c r="F23" s="53"/>
     </row>
     <row r="24" spans="1:6">
-      <c r="A24" s="54"/>
-      <c r="B24" s="54"/>
-      <c r="C24" s="54"/>
-      <c r="D24" s="54"/>
-      <c r="E24" s="54"/>
-      <c r="F24" s="54"/>
+      <c r="A24" s="53"/>
+      <c r="B24" s="53"/>
+      <c r="C24" s="53"/>
+      <c r="D24" s="53"/>
+      <c r="E24" s="53"/>
+      <c r="F24" s="53"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -3783,15 +3783,15 @@
       <c r="Q2" s="47"/>
     </row>
     <row r="3" spans="1:17" ht="15.75">
-      <c r="A3" s="48" t="s">
+      <c r="A3" s="54" t="s">
         <v>162</v>
       </c>
-      <c r="B3" s="48"/>
-      <c r="C3" s="48"/>
-      <c r="D3" s="48"/>
-      <c r="E3" s="48"/>
-      <c r="F3" s="48"/>
-      <c r="G3" s="48"/>
+      <c r="B3" s="54"/>
+      <c r="C3" s="54"/>
+      <c r="D3" s="54"/>
+      <c r="E3" s="54"/>
+      <c r="F3" s="54"/>
+      <c r="G3" s="54"/>
     </row>
     <row r="5" spans="1:17" ht="15">
       <c r="A5" s="1" t="s">
@@ -3829,7 +3829,7 @@
         <v>1.0958249999999998</v>
       </c>
       <c r="C6" s="34">
-        <f t="shared" ref="C6:C16" si="1">FC_AMT*B6</f>
+        <f>FC_AMT*B6</f>
         <v>13697812.499999998</v>
       </c>
       <c r="D6" s="34">
@@ -3841,15 +3841,15 @@
         <v>14633514.240847424</v>
       </c>
       <c r="F6" s="34">
-        <f t="shared" ref="F6:F16" si="2">FC_AMT*MAX(B6,K_PUT)-FC_AMT*PREM_PUT</f>
+        <f t="shared" ref="F6:F16" si="1">FC_AMT*MAX(B6,K_PUT)-FC_AMT*PREM_PUT</f>
         <v>14206250</v>
       </c>
       <c r="G6" s="34">
-        <f t="shared" ref="G6:G16" si="3">FC_AMT*B6+FC_AMT*MAX(B6-K_CALL,0)-FC_AMT*PREM_CALL</f>
+        <f t="shared" ref="G6:G16" si="2">FC_AMT*B6+FC_AMT*MAX(B6-K_CALL,0)-FC_AMT*PREM_CALL</f>
         <v>13422812.499999998</v>
       </c>
       <c r="H6" s="35" t="str">
-        <f t="shared" ref="H6:H16" si="4">TEXT(A6,"0%")</f>
+        <f t="shared" ref="H6:H16" si="3">TEXT(A6,"0%")</f>
         <v>95%</v>
       </c>
     </row>
@@ -3863,7 +3863,7 @@
         <v>1.1073599999999999</v>
       </c>
       <c r="C7" s="26">
-        <f t="shared" si="1"/>
+        <f t="shared" ref="C6:C16" si="4">FC_AMT*B7</f>
         <v>13841999.999999998</v>
       </c>
       <c r="D7" s="26">
@@ -3875,15 +3875,15 @@
         <v>14633514.240847424</v>
       </c>
       <c r="F7" s="26">
+        <f t="shared" si="1"/>
+        <v>14206250</v>
+      </c>
+      <c r="G7" s="26">
         <f t="shared" si="2"/>
-        <v>14206250</v>
-      </c>
-      <c r="G7" s="26">
+        <v>13566999.999999998</v>
+      </c>
+      <c r="H7" s="35" t="str">
         <f t="shared" si="3"/>
-        <v>13566999.999999998</v>
-      </c>
-      <c r="H7" s="35" t="str">
-        <f t="shared" si="4"/>
         <v>96%</v>
       </c>
     </row>
@@ -3897,7 +3897,7 @@
         <v>1.118895</v>
       </c>
       <c r="C8" s="26">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>13986187.5</v>
       </c>
       <c r="D8" s="26">
@@ -3909,15 +3909,15 @@
         <v>14633514.240847424</v>
       </c>
       <c r="F8" s="26">
+        <f t="shared" si="1"/>
+        <v>14206250</v>
+      </c>
+      <c r="G8" s="26">
         <f t="shared" si="2"/>
-        <v>14206250</v>
-      </c>
-      <c r="G8" s="26">
+        <v>13711187.5</v>
+      </c>
+      <c r="H8" s="35" t="str">
         <f t="shared" si="3"/>
-        <v>13711187.5</v>
-      </c>
-      <c r="H8" s="35" t="str">
-        <f t="shared" si="4"/>
         <v>97%</v>
       </c>
     </row>
@@ -3931,7 +3931,7 @@
         <v>1.13043</v>
       </c>
       <c r="C9" s="26">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>14130375</v>
       </c>
       <c r="D9" s="26">
@@ -3943,15 +3943,15 @@
         <v>14633514.240847424</v>
       </c>
       <c r="F9" s="26">
+        <f t="shared" si="1"/>
+        <v>14206250</v>
+      </c>
+      <c r="G9" s="26">
         <f t="shared" si="2"/>
-        <v>14206250</v>
-      </c>
-      <c r="G9" s="26">
+        <v>13855375</v>
+      </c>
+      <c r="H9" s="35" t="str">
         <f t="shared" si="3"/>
-        <v>13855375</v>
-      </c>
-      <c r="H9" s="35" t="str">
-        <f t="shared" si="4"/>
         <v>98%</v>
       </c>
     </row>
@@ -3965,7 +3965,7 @@
         <v>1.1419649999999999</v>
       </c>
       <c r="C10" s="26">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>14274562.499999998</v>
       </c>
       <c r="D10" s="26">
@@ -3977,15 +3977,15 @@
         <v>14633514.240847424</v>
       </c>
       <c r="F10" s="26">
+        <f t="shared" si="1"/>
+        <v>14206250</v>
+      </c>
+      <c r="G10" s="26">
         <f t="shared" si="2"/>
-        <v>14206250</v>
-      </c>
-      <c r="G10" s="26">
+        <v>13999562.499999998</v>
+      </c>
+      <c r="H10" s="35" t="str">
         <f t="shared" si="3"/>
-        <v>13999562.499999998</v>
-      </c>
-      <c r="H10" s="35" t="str">
-        <f t="shared" si="4"/>
         <v>99%</v>
       </c>
     </row>
@@ -3999,7 +3999,7 @@
         <v>1.1535</v>
       </c>
       <c r="C11" s="26">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>14418750</v>
       </c>
       <c r="D11" s="26">
@@ -4011,15 +4011,15 @@
         <v>14633514.240847424</v>
       </c>
       <c r="F11" s="26">
+        <f t="shared" si="1"/>
+        <v>14206250</v>
+      </c>
+      <c r="G11" s="26">
         <f t="shared" si="2"/>
-        <v>14206250</v>
-      </c>
-      <c r="G11" s="26">
+        <v>14143750</v>
+      </c>
+      <c r="H11" s="35" t="str">
         <f t="shared" si="3"/>
-        <v>14143750</v>
-      </c>
-      <c r="H11" s="35" t="str">
-        <f t="shared" si="4"/>
         <v>100%</v>
       </c>
     </row>
@@ -4033,7 +4033,7 @@
         <v>1.165035</v>
       </c>
       <c r="C12" s="26">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>14562937.5</v>
       </c>
       <c r="D12" s="26">
@@ -4045,15 +4045,15 @@
         <v>14633514.240847424</v>
       </c>
       <c r="F12" s="26">
+        <f t="shared" si="1"/>
+        <v>14350437.5</v>
+      </c>
+      <c r="G12" s="26">
         <f t="shared" si="2"/>
-        <v>14350437.5</v>
-      </c>
-      <c r="G12" s="26">
+        <v>14432125</v>
+      </c>
+      <c r="H12" s="35" t="str">
         <f t="shared" si="3"/>
-        <v>14432125</v>
-      </c>
-      <c r="H12" s="35" t="str">
-        <f t="shared" si="4"/>
         <v>101%</v>
       </c>
     </row>
@@ -4067,7 +4067,7 @@
         <v>1.1765699999999999</v>
       </c>
       <c r="C13" s="26">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>14707124.999999998</v>
       </c>
       <c r="D13" s="26">
@@ -4079,15 +4079,15 @@
         <v>14633514.240847424</v>
       </c>
       <c r="F13" s="26">
+        <f t="shared" si="1"/>
+        <v>14494624.999999998</v>
+      </c>
+      <c r="G13" s="26">
         <f t="shared" si="2"/>
-        <v>14494624.999999998</v>
-      </c>
-      <c r="G13" s="26">
+        <v>14720499.999999996</v>
+      </c>
+      <c r="H13" s="35" t="str">
         <f t="shared" si="3"/>
-        <v>14720499.999999996</v>
-      </c>
-      <c r="H13" s="35" t="str">
-        <f t="shared" si="4"/>
         <v>102%</v>
       </c>
     </row>
@@ -4101,7 +4101,7 @@
         <v>1.188105</v>
       </c>
       <c r="C14" s="26">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>14851312.5</v>
       </c>
       <c r="D14" s="26">
@@ -4113,15 +4113,15 @@
         <v>14633514.240847424</v>
       </c>
       <c r="F14" s="26">
+        <f t="shared" si="1"/>
+        <v>14638812.5</v>
+      </c>
+      <c r="G14" s="26">
         <f t="shared" si="2"/>
-        <v>14638812.5</v>
-      </c>
-      <c r="G14" s="26">
+        <v>15008875</v>
+      </c>
+      <c r="H14" s="35" t="str">
         <f t="shared" si="3"/>
-        <v>15008875</v>
-      </c>
-      <c r="H14" s="35" t="str">
-        <f t="shared" si="4"/>
         <v>103%</v>
       </c>
     </row>
@@ -4135,7 +4135,7 @@
         <v>1.19964</v>
       </c>
       <c r="C15" s="26">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>14995500</v>
       </c>
       <c r="D15" s="26">
@@ -4147,15 +4147,15 @@
         <v>14633514.240847424</v>
       </c>
       <c r="F15" s="26">
+        <f t="shared" si="1"/>
+        <v>14783000</v>
+      </c>
+      <c r="G15" s="26">
         <f t="shared" si="2"/>
-        <v>14783000</v>
-      </c>
-      <c r="G15" s="26">
+        <v>15297250</v>
+      </c>
+      <c r="H15" s="35" t="str">
         <f t="shared" si="3"/>
-        <v>15297250</v>
-      </c>
-      <c r="H15" s="35" t="str">
-        <f t="shared" si="4"/>
         <v>104%</v>
       </c>
     </row>
@@ -4169,7 +4169,7 @@
         <v>1.2111750000000001</v>
       </c>
       <c r="C16" s="26">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>15139687.500000002</v>
       </c>
       <c r="D16" s="26">
@@ -4181,15 +4181,15 @@
         <v>14633514.240847424</v>
       </c>
       <c r="F16" s="26">
+        <f t="shared" si="1"/>
+        <v>14927187.500000002</v>
+      </c>
+      <c r="G16" s="26">
         <f t="shared" si="2"/>
-        <v>14927187.500000002</v>
-      </c>
-      <c r="G16" s="26">
+        <v>15585625.000000004</v>
+      </c>
+      <c r="H16" s="35" t="str">
         <f t="shared" si="3"/>
-        <v>15585625.000000004</v>
-      </c>
-      <c r="H16" s="35" t="str">
-        <f t="shared" si="4"/>
         <v>105%</v>
       </c>
     </row>

</xml_diff>